<commit_message>
Plate designer: the control file format is no longer fixed per run
Column names are read by meaning (replicates, n_wells, wells/plate, priority,
seq), well counts run 0-96 instead of stopping at four, and a control type the
tool has never heard of is accepted on a control sheet while a patient specimen
type is still refused. The sized control area is cut from whole control chunks so
it works at any well count, and the plate count it promises is counted from the
chunks autofill can cut rather than divided out of 96.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QBH1P2zpiSLx4BR7WKjhzK
</commit_message>
<xml_diff>
--- a/PhIPSeq_Control_Template_v1.xlsx
+++ b/PhIPSeq_Control_Template_v1.xlsx
@@ -522,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:D35"/>
+  <dimension ref="B2:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="2" max="2"/>
@@ -585,53 +585,43 @@
     <row r="10">
       <c r="B10" s="2" t="inlineStr">
         <is>
+          <t>Column names are read by meaning, so this run’s file can say replicates, n_wells or wells/plate instead of wells_per_plate, and priority or seq instead of order. Nothing here is fixed for every run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="2" t="inlineStr">
+        <is>
           <t>Set wells_per_plate to 0 to import a control without putting it in the layout — useful for one you keep on hand but are not running this time.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="B12" s="4" t="inlineStr">
+    <row r="13">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Column</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>What it is</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>Required?</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>sample_id</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Your name for the control. Appears in the Lab Plate Maps. Must be unique in this file.</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Required</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>sample_type</t>
+          <t>sample_id</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>mAb, control, or assay control. Anything else is refused: a patient sample in a control file is the wrong file.</t>
+          <t>Your name for the control. Appears in the Lab Plate Maps. Must be unique in this file.</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -643,46 +633,46 @@
     <row r="15">
       <c r="B15" s="3" t="inlineStr">
         <is>
+          <t>sample_type</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Any control type, including one of your own. Recognised specimen types (serum, plasma, whole blood, CSF) are refused — a patient sample in a control file is the wrong file.</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="3" t="inlineStr">
+        <is>
           <t>wells_per_plate</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>How many wells this control takes on EVERY plate, 0-4.</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>How many wells this control takes on EVERY plate. Any count the control area can hold.</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Required</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>order</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Order within the control area, lowest first. Blank falls back to row order.</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Recommended</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>cohort</t>
+          <t>order</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Grouping and colour, e.g. "Lab controls". Controls are never auto-filled, so this only affects how they read.</t>
+          <t>Order within the control area, lowest first. Blank falls back to row order. Also read from priority, sort_order, seq.</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -694,12 +684,12 @@
     <row r="18">
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>volume_mL</t>
+          <t>cohort</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Volume on hand, for the volume pre-flight check.</t>
+          <t>Grouping and colour, e.g. "Lab controls". Controls are never auto-filled, so this only affects how they read.</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -711,29 +701,29 @@
     <row r="19">
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>min_volume_required_mL</t>
+          <t>volume_mL</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Per-control override of the volume floor.</t>
+          <t>Volume on hand, for the volume pre-flight check.</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Recommended</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>repeat_across_plates</t>
+          <t>min_volume_required_mL</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>"all"/"yes", or a plate list such as 1,3,5. Marks a bridging control.</t>
+          <t>Per-control override of the volume floor.</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -745,12 +735,12 @@
     <row r="21">
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>source_rack / source_position</t>
+          <t>repeat_across_plates</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Where the tube sits, for the worklist and Tecan exports.</t>
+          <t>"all"/"yes", or a plate list such as 1,3,5. Marks a bridging control.</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -762,12 +752,12 @@
     <row r="22">
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>subject_id</t>
+          <t>source_rack / source_position</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Usually blank for a control. If given, tiu_id becomes sample_id_subject_id.</t>
+          <t>Where the tube sits, for the worklist and Tecan exports.</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -779,32 +769,41 @@
     <row r="23">
       <c r="B23" s="2" t="inlineStr">
         <is>
+          <t>subject_id</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Usually blank for a control. If given, tiu_id becomes sample_id_subject_id.</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="2" t="inlineStr">
+        <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>Anything else — lot number, catalogue number, supplier. Carried into the export.</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="B25" s="3" t="inlineStr">
+    <row r="26">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>What the designer does with it</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" s="2" t="inlineStr"/>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Rows are merged into the sample pool as controls, so the control template can place them.</t>
         </is>
       </c>
     </row>
@@ -812,7 +811,7 @@
       <c r="B27" s="2" t="inlineStr"/>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>A row that is not a control type is refused and named, rather than quietly added.</t>
+          <t>Rows are merged into the sample pool as controls, so the control template can place them.</t>
         </is>
       </c>
     </row>
@@ -820,7 +819,7 @@
       <c r="B28" s="2" t="inlineStr"/>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Re-importing the same file does not duplicate: rows already present are left alone.</t>
+          <t>A control type this tool has never heard of is accepted and reported. A patient specimen type is refused and named.</t>
         </is>
       </c>
     </row>
@@ -828,7 +827,7 @@
       <c r="B29" s="2" t="inlineStr"/>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Imported controls are written into the exported Input Samples sheet with a note naming this file, so the exported manifest still re-opens on its own.</t>
+          <t>Re-importing the same file does not duplicate: rows already present are left alone.</t>
         </is>
       </c>
     </row>
@@ -836,36 +835,44 @@
       <c r="B30" s="2" t="inlineStr"/>
       <c r="C30" s="2" t="inlineStr">
         <is>
+          <t>Imported controls are written into the exported Input Samples sheet with a note naming this file, so the exported manifest still re-opens on its own.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="2" t="inlineStr"/>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
           <t>Controls are never auto-filled. They are stamped into the reserved control area.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="B32" s="3" t="inlineStr">
+    <row r="33">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>Colour Legend</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="B33" s="5" t="inlineStr"/>
-      <c r="C33" s="6" t="inlineStr">
+    <row r="34">
+      <c r="B34" s="5" t="inlineStr"/>
+      <c r="C34" s="6" t="inlineStr">
         <is>
           <t>Yellow = you fill this in</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="B34" s="7" t="inlineStr"/>
-      <c r="C34" s="6" t="inlineStr">
+    <row r="35">
+      <c r="B35" s="7" t="inlineStr"/>
+      <c r="C35" s="6" t="inlineStr">
         <is>
           <t>Blue italic row 2 = example, delete before uploading</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="B35" s="8" t="inlineStr"/>
-      <c r="C35" s="6" t="inlineStr">
+    <row r="36">
+      <c r="B36" s="8" t="inlineStr"/>
+      <c r="C36" s="6" t="inlineStr">
         <is>
           <t>Red = a required value is missing on a row that has other data</t>
         </is>
@@ -1588,12 +1595,12 @@
     <dataValidation sqref="A3:A41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="sample_id" error="sample_id is required and must be unique within this file. It is how the control is named on the Lab Plate Maps." type="custom">
       <formula1>=AND(LEN(TRIM($A3))&gt;0,COUNTIF($A$3:$A$41,$A3)&lt;=1)</formula1>
     </dataValidation>
-    <dataValidation sqref="B3:B41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="sample_type" error="A control file holds control types only: mAb, control or assay control. Anything else is refused on import." type="list">
+    <dataValidation sqref="B3:B41" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="sample_type" prompt="Pick one, or type your own — a pooled reference, an IVIG standard, a titration ladder. Any type the designer does not recognise is taken as a control. Do not put a specimen type here (serum, plasma, whole blood, CSF): those are refused, because that is how a sample manifest gets loaded as a control file by mistake." type="list">
       <formula1>"mAb,control,assay control"</formula1>
     </dataValidation>
-    <dataValidation sqref="C3:C41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="wells_per_plate" error="How many wells this control takes on EVERY plate, 0 to 4. 0 imports the control but leaves it out of the layout." type="whole" operator="between">
+    <dataValidation sqref="C3:C41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="wells_per_plate" error="How many wells this control takes on EVERY plate. A plate holds 96, and the control area has to be big enough — the designer checks the fit and can size the area to this file. 0 imports the control but leaves it out of the layout." type="whole" operator="between">
       <formula1>0</formula1>
-      <formula2>4</formula2>
+      <formula2>96</formula2>
     </dataValidation>
     <dataValidation sqref="D3:D41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="order" error="The order controls are laid into the control area, lowest first. Leave blank to use the row order." type="whole" operator="between">
       <formula1>1</formula1>

</xml_diff>